<commit_message>
Key rides the Slivo Scramble header — the only senior-tees event
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/locigno-outing.xlsx
+++ b/assets/locigno-outing.xlsx
@@ -697,29 +697,29 @@
           <t xml:space="preserve">Shawn McWilliams</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr" s="7">
+      <c r="D5" t="inlineStr">
         <is>
           <t xml:space="preserve">Bud Deflorio</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr" s="7">
+      <c r="A6" t="inlineStr">
         <is>
           <t xml:space="preserve">Frank Skully</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr" s="7">
+      <c r="B6" t="inlineStr">
         <is>
           <t xml:space="preserve">George Hahn</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr" s="7">
+      <c r="C6" t="inlineStr">
         <is>
           <t xml:space="preserve">Don Andrews</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr" s="7">
+      <c r="D6" t="inlineStr">
         <is>
           <t xml:space="preserve">Bret Traylor</t>
         </is>
@@ -758,12 +758,12 @@
           <t xml:space="preserve">Jeff Myers Jr.</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr" s="7">
+      <c r="C8" t="inlineStr">
         <is>
           <t xml:space="preserve">Dave Powers</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr" s="7">
+      <c r="D8" t="inlineStr">
         <is>
           <t xml:space="preserve">John Locigno</t>
         </is>
@@ -785,19 +785,19 @@
           <t xml:space="preserve">John Baucco</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr" s="7">
+      <c r="D9" t="inlineStr">
         <is>
           <t xml:space="preserve">JAM</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr" s="7">
+      <c r="A10" t="inlineStr">
         <is>
           <t xml:space="preserve">Joe Locigno</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr" s="7">
+      <c r="B10" t="inlineStr">
         <is>
           <t xml:space="preserve">Pat Bruckman</t>
         </is>
@@ -1051,17 +1051,17 @@
           <t xml:space="preserve">Ryan Weed</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr" s="7">
+      <c r="B25" t="inlineStr">
         <is>
           <t xml:space="preserve">Frank Skully</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr" s="7">
+      <c r="C25" t="inlineStr">
         <is>
           <t xml:space="preserve">Pat Bruckman</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr" s="7">
+      <c r="D25" t="inlineStr">
         <is>
           <t xml:space="preserve">George Hahn</t>
         </is>
@@ -1122,12 +1122,12 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr" s="7">
+      <c r="A28" t="inlineStr">
         <is>
           <t xml:space="preserve">Joe Locigno</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr" s="7">
+      <c r="B28" t="inlineStr">
         <is>
           <t xml:space="preserve">Bud Deflorio</t>
         </is>
@@ -1154,12 +1154,12 @@
           <t xml:space="preserve">Chris Palmeri</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr" s="7">
+      <c r="C29" t="inlineStr">
         <is>
           <t xml:space="preserve">Dave Powers</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr" s="7">
+      <c r="D29" t="inlineStr">
         <is>
           <t xml:space="preserve">John Locigno</t>
         </is>
@@ -1171,7 +1171,7 @@
           <t xml:space="preserve">Ryan Miers</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr" s="7">
+      <c r="B30" t="inlineStr">
         <is>
           <t xml:space="preserve">Don Andrews</t>
         </is>
@@ -1181,7 +1181,7 @@
           <t xml:space="preserve">Nate Stevens</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr" s="7">
+      <c r="D30" t="inlineStr">
         <is>
           <t xml:space="preserve">JAM</t>
         </is>
@@ -1198,7 +1198,7 @@
           <t xml:space="preserve">Mike Bregitzer</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr" s="7">
+      <c r="C31" t="inlineStr">
         <is>
           <t xml:space="preserve">Bret Traylor</t>
         </is>
@@ -1233,7 +1233,7 @@
           <t xml:space="preserve">Ryan Weed</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr" s="7">
+      <c r="B34" t="inlineStr">
         <is>
           <t xml:space="preserve">Bud Deflorio</t>
         </is>
@@ -1255,7 +1255,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr" s="7">
+      <c r="A35" t="inlineStr">
         <is>
           <t xml:space="preserve">Joe Locigno</t>
         </is>
@@ -1265,12 +1265,12 @@
           <t xml:space="preserve">Alan Scott</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr" s="7">
+      <c r="C35" t="inlineStr">
         <is>
           <t xml:space="preserve">Dave Powers</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr" s="7">
+      <c r="D35" t="inlineStr">
         <is>
           <t xml:space="preserve">George Hahn</t>
         </is>
@@ -1287,12 +1287,12 @@
           <t xml:space="preserve">Shawn McWilliams</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr" s="7">
+      <c r="B36" t="inlineStr">
         <is>
           <t xml:space="preserve">Don Andrews</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr" s="7">
+      <c r="C36" t="inlineStr">
         <is>
           <t xml:space="preserve">Pat Bruckman</t>
         </is>
@@ -1319,7 +1319,7 @@
           <t xml:space="preserve">Jason Salerno</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr" s="7">
+      <c r="D37" t="inlineStr">
         <is>
           <t xml:space="preserve">John Locigno</t>
         </is>
@@ -1353,17 +1353,17 @@
           <t xml:space="preserve">Zeke Deflorio</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr" s="7">
+      <c r="B39" t="inlineStr">
         <is>
           <t xml:space="preserve">Frank Skully</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr" s="7">
+      <c r="C39" t="inlineStr">
         <is>
           <t xml:space="preserve">Bret Traylor</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr" s="7">
+      <c r="D39" t="inlineStr">
         <is>
           <t xml:space="preserve">JAM</t>
         </is>

</xml_diff>